<commit_message>
Datasets de BCS, Hidalgo, Nayarit y SLP
</commit_message>
<xml_diff>
--- a/datasets/20261021_recontrataciones_sonora.xlsx
+++ b/datasets/20261021_recontrataciones_sonora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inemexico-my.sharepoint.com/personal/jannet_piteros_ine_mx/Documents/1. PROCESO ELECTORAL 2027/SE y CAE/Recontratación SE y CAE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{9E3F16FB-CB26-4EE7-8B51-72B5D2FB9592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27763F04-7694-4881-8377-B22251C958C1}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{9E3F16FB-CB26-4EE7-8B51-72B5D2FB9592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B1E0346-557C-4A7B-B6C2-D40485889232}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D3C7E6B5-2A0E-4AF2-BE80-0C96F41EC4B0}"/>
   </bookViews>
@@ -264,7 +264,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -283,6 +283,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="31">
     <border>
@@ -690,7 +696,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -773,8 +779,47 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -794,21 +839,6 @@
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -821,28 +851,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1266,50 +1278,50 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.3">
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="31"/>
-      <c r="Q2" s="31"/>
-      <c r="R2" s="31"/>
-      <c r="S2" s="31"/>
-      <c r="T2" s="31"/>
-      <c r="U2" s="31"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="44"/>
+      <c r="Q2" s="44"/>
+      <c r="R2" s="44"/>
+      <c r="S2" s="44"/>
+      <c r="T2" s="44"/>
+      <c r="U2" s="44"/>
     </row>
     <row r="3" spans="2:21" s="2" customFormat="1" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="C3" s="32" t="s">
+      <c r="C3" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32"/>
-      <c r="M3" s="32"/>
-      <c r="N3" s="32"/>
-      <c r="O3" s="32"/>
-      <c r="P3" s="32"/>
-      <c r="Q3" s="32"/>
-      <c r="R3" s="32"/>
-      <c r="S3" s="32"/>
-      <c r="T3" s="32"/>
-      <c r="U3" s="32"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="45"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="45"/>
+      <c r="L3" s="45"/>
+      <c r="M3" s="45"/>
+      <c r="N3" s="45"/>
+      <c r="O3" s="45"/>
+      <c r="P3" s="45"/>
+      <c r="Q3" s="45"/>
+      <c r="R3" s="45"/>
+      <c r="S3" s="45"/>
+      <c r="T3" s="45"/>
+      <c r="U3" s="45"/>
     </row>
     <row r="4" spans="2:21" s="2" customFormat="1" ht="20.25" x14ac:dyDescent="0.3">
       <c r="C4" s="1"/>
@@ -1333,135 +1345,135 @@
       <c r="U4" s="1"/>
     </row>
     <row r="5" spans="2:21" s="2" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="C5" s="45" t="s">
+      <c r="C5" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="45"/>
-      <c r="I5" s="45"/>
-      <c r="J5" s="45"/>
-      <c r="K5" s="45"/>
-      <c r="L5" s="45"/>
-      <c r="M5" s="45"/>
-      <c r="N5" s="45"/>
-      <c r="O5" s="45"/>
-      <c r="P5" s="45"/>
-      <c r="Q5" s="45"/>
-      <c r="R5" s="45"/>
-      <c r="S5" s="45"/>
+      <c r="D5" s="53"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53"/>
+      <c r="G5" s="53"/>
+      <c r="H5" s="53"/>
+      <c r="I5" s="53"/>
+      <c r="J5" s="53"/>
+      <c r="K5" s="53"/>
+      <c r="L5" s="53"/>
+      <c r="M5" s="53"/>
+      <c r="N5" s="53"/>
+      <c r="O5" s="53"/>
+      <c r="P5" s="53"/>
+      <c r="Q5" s="53"/>
+      <c r="R5" s="53"/>
+      <c r="S5" s="53"/>
       <c r="T5" s="7"/>
       <c r="U5" s="7"/>
     </row>
     <row r="6" spans="2:21" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="46"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="46"/>
-      <c r="J6" s="46"/>
-      <c r="K6" s="46"/>
-      <c r="L6" s="46"/>
-      <c r="M6" s="46"/>
-      <c r="N6" s="46"/>
-      <c r="O6" s="46"/>
-      <c r="P6" s="46"/>
-      <c r="Q6" s="46"/>
-      <c r="R6" s="46"/>
-      <c r="S6" s="46"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="31"/>
+      <c r="L6" s="31"/>
+      <c r="M6" s="31"/>
+      <c r="N6" s="31"/>
+      <c r="O6" s="31"/>
+      <c r="P6" s="31"/>
+      <c r="Q6" s="31"/>
+      <c r="R6" s="31"/>
+      <c r="S6" s="31"/>
       <c r="T6" s="8"/>
       <c r="U6" s="8"/>
     </row>
     <row r="7" spans="2:21" s="2" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
     </row>
     <row r="8" spans="2:21" s="2" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="41"/>
-      <c r="D8" s="47">
+      <c r="C8" s="33"/>
+      <c r="D8" s="34">
         <v>46315</v>
       </c>
-      <c r="E8" s="48"/>
-      <c r="F8" s="48"/>
-      <c r="G8" s="49"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="36"/>
     </row>
     <row r="9" spans="2:21" s="2" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="52" t="s">
+      <c r="B9" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="52"/>
-      <c r="D9" s="52"/>
-      <c r="E9" s="52"/>
-      <c r="F9" s="52"/>
-      <c r="G9" s="52"/>
-      <c r="H9" s="52"/>
-      <c r="I9" s="52"/>
-      <c r="J9" s="52"/>
-      <c r="K9" s="52"/>
-      <c r="L9" s="52"/>
-      <c r="M9" s="52"/>
-      <c r="N9" s="52"/>
-      <c r="O9" s="52"/>
-      <c r="P9" s="52"/>
-      <c r="Q9" s="52"/>
-      <c r="R9" s="52"/>
-      <c r="S9" s="52"/>
-      <c r="T9" s="52"/>
-      <c r="U9" s="52"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
+      <c r="H9" s="43"/>
+      <c r="I9" s="43"/>
+      <c r="J9" s="43"/>
+      <c r="K9" s="43"/>
+      <c r="L9" s="43"/>
+      <c r="M9" s="43"/>
+      <c r="N9" s="43"/>
+      <c r="O9" s="43"/>
+      <c r="P9" s="43"/>
+      <c r="Q9" s="43"/>
+      <c r="R9" s="43"/>
+      <c r="S9" s="43"/>
+      <c r="T9" s="43"/>
+      <c r="U9" s="43"/>
     </row>
     <row r="10" spans="2:21" s="2" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="30" t="s">
+      <c r="B10" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="C10" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="D10" s="44" t="s">
+      <c r="D10" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="33" t="s">
+      <c r="E10" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="35" t="s">
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="47"/>
+      <c r="J10" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="K10" s="36"/>
-      <c r="L10" s="36"/>
-      <c r="M10" s="36"/>
-      <c r="N10" s="36"/>
-      <c r="O10" s="42" t="s">
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
+      <c r="M10" s="49"/>
+      <c r="N10" s="49"/>
+      <c r="O10" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="P10" s="34"/>
-      <c r="Q10" s="34"/>
-      <c r="R10" s="34"/>
-      <c r="S10" s="43"/>
-      <c r="T10" s="30" t="s">
+      <c r="P10" s="47"/>
+      <c r="Q10" s="47"/>
+      <c r="R10" s="47"/>
+      <c r="S10" s="51"/>
+      <c r="T10" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="U10" s="30" t="s">
+      <c r="U10" s="32" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="2:21" s="2" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="30"/>
-      <c r="C11" s="30"/>
-      <c r="D11" s="44"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="52"/>
       <c r="E11" s="37" t="s">
         <v>12</v>
       </c>
@@ -1477,19 +1489,19 @@
       <c r="I11" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="39" t="s">
+      <c r="J11" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="K11" s="39" t="s">
+      <c r="K11" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="L11" s="39" t="s">
+      <c r="L11" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="M11" s="39" t="s">
+      <c r="M11" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="N11" s="39" t="s">
+      <c r="N11" s="41" t="s">
         <v>16</v>
       </c>
       <c r="O11" s="37" t="s">
@@ -1504,11 +1516,11 @@
       <c r="R11" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="S11" s="50" t="s">
+      <c r="S11" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="T11" s="30"/>
-      <c r="U11" s="30"/>
+      <c r="T11" s="32"/>
+      <c r="U11" s="32"/>
     </row>
     <row r="12" spans="2:21" s="3" customFormat="1" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="11" t="s">
@@ -1517,24 +1529,24 @@
       <c r="C12" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="44"/>
+      <c r="D12" s="52"/>
       <c r="E12" s="38"/>
       <c r="F12" s="38"/>
       <c r="G12" s="38"/>
       <c r="H12" s="38"/>
       <c r="I12" s="38"/>
-      <c r="J12" s="40"/>
-      <c r="K12" s="40"/>
-      <c r="L12" s="40"/>
-      <c r="M12" s="40"/>
-      <c r="N12" s="40"/>
+      <c r="J12" s="42"/>
+      <c r="K12" s="42"/>
+      <c r="L12" s="42"/>
+      <c r="M12" s="42"/>
+      <c r="N12" s="42"/>
       <c r="O12" s="38"/>
       <c r="P12" s="38"/>
       <c r="Q12" s="38"/>
       <c r="R12" s="38"/>
-      <c r="S12" s="51"/>
-      <c r="T12" s="30"/>
-      <c r="U12" s="30"/>
+      <c r="S12" s="40"/>
+      <c r="T12" s="32"/>
+      <c r="U12" s="32"/>
     </row>
     <row r="13" spans="2:21" s="2" customFormat="1" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="10">
@@ -1573,7 +1585,7 @@
       <c r="M13" s="10">
         <v>3</v>
       </c>
-      <c r="N13" s="12">
+      <c r="N13" s="14">
         <v>0</v>
       </c>
       <c r="O13" s="17" t="s">
@@ -1592,6 +1604,7 @@
         <v>11</v>
       </c>
       <c r="T13" s="18">
+        <f>J13+E13</f>
         <v>137</v>
       </c>
       <c r="U13" s="14"/>
@@ -1603,10 +1616,10 @@
       <c r="C14" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="53">
+      <c r="E14" s="30">
         <v>40</v>
       </c>
       <c r="F14" s="10">
@@ -1622,15 +1635,15 @@
         <v>0</v>
       </c>
       <c r="J14" s="28">
-        <v>81</v>
-      </c>
-      <c r="K14" s="10">
+        <v>82</v>
+      </c>
+      <c r="K14" s="54">
         <v>77</v>
       </c>
-      <c r="L14" s="10">
+      <c r="L14" s="54">
         <v>4</v>
       </c>
-      <c r="M14" s="10">
+      <c r="M14" s="54">
         <v>1</v>
       </c>
       <c r="N14" s="14">
@@ -1652,7 +1665,8 @@
         <v>11</v>
       </c>
       <c r="T14" s="18">
-        <v>81</v>
+        <f t="shared" ref="T14:T19" si="0">J14+E14</f>
+        <v>122</v>
       </c>
       <c r="U14" s="18"/>
     </row>
@@ -1693,7 +1707,7 @@
       <c r="M15" s="10">
         <v>2</v>
       </c>
-      <c r="N15" s="12">
+      <c r="N15" s="14">
         <v>0</v>
       </c>
       <c r="O15" s="15" t="s">
@@ -1712,6 +1726,7 @@
         <v>11</v>
       </c>
       <c r="T15" s="18">
+        <f t="shared" si="0"/>
         <v>110</v>
       </c>
       <c r="U15" s="18"/>
@@ -1753,7 +1768,7 @@
       <c r="M16" s="10">
         <v>7</v>
       </c>
-      <c r="N16" s="12">
+      <c r="N16" s="14">
         <v>0</v>
       </c>
       <c r="O16" s="13" t="s">
@@ -1771,7 +1786,8 @@
       <c r="S16" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="T16" s="12">
+      <c r="T16" s="18">
+        <f t="shared" si="0"/>
         <v>131</v>
       </c>
       <c r="U16" s="18"/>
@@ -1831,8 +1847,8 @@
       <c r="S17" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="T17" s="14">
-        <f>SUM(E17,J17,O17)</f>
+      <c r="T17" s="18">
+        <f t="shared" si="0"/>
         <v>158</v>
       </c>
       <c r="U17" s="18"/>
@@ -1894,6 +1910,7 @@
         <v>11</v>
       </c>
       <c r="T18" s="18">
+        <f t="shared" si="0"/>
         <v>151</v>
       </c>
       <c r="U18" s="22"/>
@@ -1909,31 +1926,31 @@
         <v>24</v>
       </c>
       <c r="E19" s="15">
-        <v>22</v>
-      </c>
-      <c r="F19" s="10">
+        <v>50</v>
+      </c>
+      <c r="F19" s="55">
         <v>10</v>
       </c>
-      <c r="G19" s="10">
+      <c r="G19" s="55">
         <v>7</v>
       </c>
-      <c r="H19" s="10">
-        <v>32</v>
+      <c r="H19" s="55">
+        <v>33</v>
       </c>
       <c r="I19" s="14">
         <v>0</v>
       </c>
-      <c r="J19" s="13">
-        <v>50</v>
+      <c r="J19" s="55">
+        <v>57</v>
       </c>
       <c r="K19" s="10">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L19" s="10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M19" s="10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N19" s="14">
         <v>0</v>
@@ -1954,7 +1971,8 @@
         <v>11</v>
       </c>
       <c r="T19" s="18">
-        <v>72</v>
+        <f t="shared" si="0"/>
+        <v>107</v>
       </c>
       <c r="U19" s="14"/>
     </row>
@@ -2774,6 +2792,21 @@
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="C2:U2"/>
+    <mergeCell ref="C3:U3"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="E10:I10"/>
+    <mergeCell ref="J10:N10"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="P11:P12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="O10:S10"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="Q11:Q12"/>
+    <mergeCell ref="R11:R12"/>
+    <mergeCell ref="C5:S5"/>
     <mergeCell ref="C6:S6"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="B8:C8"/>
@@ -2790,25 +2823,10 @@
     <mergeCell ref="B9:U9"/>
     <mergeCell ref="T10:T12"/>
     <mergeCell ref="U10:U12"/>
-    <mergeCell ref="C2:U2"/>
-    <mergeCell ref="C3:U3"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="E10:I10"/>
-    <mergeCell ref="J10:N10"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="P11:P12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="O10:S10"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="Q11:Q12"/>
-    <mergeCell ref="R11:R12"/>
-    <mergeCell ref="C5:S5"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="78" fitToHeight="0" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="78" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>